<commit_message>
LDF discussion piece: linkage scale and the officer hollow middle
Page 1 replaces the binary MANDATED? boxes with a career-linkage scale
(formally mandated, functionally required, expected, self-selected,
unconnected) and a four-segment meter per box, segments outlined where a
policy check is still owed. Page 2 is rebuilt as the officer development
gap: the continuum drawn horizontally in five stages with a band whose
thickness is the linkage level, so the waist at CAPT to MAJ is visible;
soldier strip for contrast; the mechanism statement; history as context;
COMDT's question with the revised IF NO wording.

Design note rewritten around the scale and the shape of the gap, with
the transcript named as the governing evidence base. Register category
Mandate becomes Career linkage (IDs -LINK) with the level recorded.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LgFPs3fMSncBgbYQ3PfA3o
</commit_message>
<xml_diff>
--- a/output/ldf-alignment-data-required.xlsx
+++ b/output/ldf-alignment-data-required.xlsx
@@ -56,7 +56,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -76,6 +76,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFBEA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CDD2B7"/>
       </patternFill>
     </fill>
     <fill>
@@ -110,7 +115,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -125,6 +130,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -641,7 +649,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>T1-O-DEVE</t>
+          <t>T1-O-DEV</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -696,7 +704,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>T1-O-MAND</t>
+          <t>T1-O-LINK</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -721,12 +729,12 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Mandate</t>
+          <t>Career linkage</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Is that development a prerequisite for promotion, embedded in the promotion course, expected but not mandatory, or unconnected?</t>
+          <t>Where does the link between the development and the transition sit: 4 formally mandated (in policy or embedded in the qualifying course), 3 functionally required (policed, not in policy), 2 expected (self-selected, high uptake), 1 self-selected (uptake by inclination), 0 unconnected?</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -736,7 +744,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>Meeting 9 Sep: Embedded: qualifying on NZCC qualifies both LDS and ELDA Lead Teams.</t>
+          <t>Meeting 9 Sep: Level 4, formally mandated: embedded in NZCC; qualifying on NZCC qualifies both LDS and ELDA Lead Teams.</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
@@ -806,7 +814,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>T1-R-DEVE</t>
+          <t>T1-R-DEV</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -861,7 +869,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>T1-R-MAND</t>
+          <t>T1-R-LINK</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -886,12 +894,12 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Mandate</t>
+          <t>Career linkage</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Is that development a prerequisite for promotion, embedded in the promotion course, expected but not mandatory, or unconnected?</t>
+          <t>Where does the link between the development and the transition sit: 4 formally mandated (in policy or embedded in the qualifying course), 3 functionally required (policed, not in policy), 2 expected (self-selected, high uptake), 1 self-selected (uptake by inclination), 0 unconnected?</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -901,7 +909,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Meeting 9 Sep: Mandated for PTE to LCPL as an included course within the JNCO course.</t>
+          <t>Meeting 9 Sep: Level 4, formally mandated: an included course within the JNCO course for PTE to LCPL.</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
@@ -971,7 +979,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>T2-O-DEVE</t>
+          <t>T2-O-DEV</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1026,7 +1034,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>T2-O-MAND</t>
+          <t>T2-O-LINK</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1051,12 +1059,12 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Mandate</t>
+          <t>Career linkage</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Is that development a prerequisite for promotion, embedded in the promotion course, expected but not mandatory, or unconnected?</t>
+          <t>Where does the link between the development and the transition sit: 4 formally mandated (in policy or embedded in the qualifying course), 3 functionally required (policed, not in policy), 2 expected (self-selected, high uptake), 1 self-selected (uptake by inclination), 0 unconnected?</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1066,12 +1074,12 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Meeting 9 Sep: Recommended, not mandated in promotion policy. Policed in function by OCS and COs: no 2LT or LT promotes to CAPT without it in practice. The single most important cell: confirm against promotion policy.</t>
-        </is>
-      </c>
-      <c r="J10" s="3" t="inlineStr">
-        <is>
-          <t>STATED 9 SEP</t>
+          <t>Meeting 9 Sep: Level 3, functionally required: not in promotion policy, but policed by OCS and COs so that no 2LT or LT promotes to CAPT without it in practice. The single most important cell: confirm the policy position.</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>TO CONFIRM</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr"/>
@@ -1136,7 +1144,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>T2-R-DEVE</t>
+          <t>T2-R-DEV</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -1191,7 +1199,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>T2-R-MAND</t>
+          <t>T2-R-LINK</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -1216,12 +1224,12 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Mandate</t>
+          <t>Career linkage</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Is that development a prerequisite for promotion, embedded in the promotion course, expected but not mandatory, or unconnected?</t>
+          <t>Where does the link between the development and the transition sit: 4 formally mandated (in policy or embedded in the qualifying course), 3 functionally required (policed, not in policy), 2 expected (self-selected, high uptake), 1 self-selected (uptake by inclination), 0 unconnected?</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1231,7 +1239,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Meeting 9 Sep: Mandated in promotion policy: CPL promoting to SGT must complete the SNCO course, which carries it. 'Very clear on the NCO front.'</t>
+          <t>Meeting 9 Sep: Level 4, formally mandated in promotion policy: CPL promoting to SGT must complete the SNCO course, which carries it. 'Very clear on the NCO front.'</t>
         </is>
       </c>
       <c r="J13" s="3" t="inlineStr">
@@ -1301,7 +1309,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>T3-O-DEVE</t>
+          <t>T3-O-DEV</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1356,7 +1364,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>T3-O-MAND</t>
+          <t>T3-O-LINK</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -1381,12 +1389,12 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Mandate</t>
+          <t>Career linkage</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Is that development a prerequisite for promotion, embedded in the promotion course, expected but not mandatory, or unconnected?</t>
+          <t>Where does the link between the development and the transition sit: 4 formally mandated (in policy or embedded in the qualifying course), 3 functionally required (policed, not in policy), 2 expected (self-selected, high uptake), 1 self-selected (uptake by inclination), 0 unconnected?</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1396,7 +1404,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Meeting 9 Sep: Neither ELDA Lead Systems nor ILD LDS Lead Systems is mandated; neither is policed in function; uptake self-selecting. Confirm against promotion policy.</t>
+          <t>Meeting 9 Sep: Level 1, self-selected: neither ELDA Lead Systems nor ILD LDS Lead Systems is mandated or policed; uptake rests on inclination. The weakest point on either continuum.</t>
         </is>
       </c>
       <c r="J16" s="3" t="inlineStr">
@@ -1466,7 +1474,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>T3-R-DEVE</t>
+          <t>T3-R-DEV</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -1521,7 +1529,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>T3-R-MAND</t>
+          <t>T3-R-LINK</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -1546,12 +1554,12 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Mandate</t>
+          <t>Career linkage</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Is that development a prerequisite for promotion, embedded in the promotion course, expected but not mandatory, or unconnected?</t>
+          <t>Where does the link between the development and the transition sit: 4 formally mandated (in policy or embedded in the qualifying course), 3 functionally required (policed, not in policy), 2 expected (self-selected, high uptake), 1 self-selected (uptake by inclination), 0 unconnected?</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1561,12 +1569,12 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Meeting 9 Sep: ELDA Lead Systems mandated on the WO course. Whether ILD LDS Lead Systems is a prerequisite for WO2: understanding is yes, with a question mark. Dave to check the promotion-course CDS.</t>
-        </is>
-      </c>
-      <c r="J19" s="3" t="inlineStr">
-        <is>
-          <t>STATED 9 SEP</t>
+          <t>Meeting 9 Sep: Level 4 for ELDA Lead Systems (mandated on the WO course). ILD LDS Lead Systems as a WO2 prerequisite: 'understanding is yes', with a question mark. Dave to check the promotion-course CDS.</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>TO CONFIRM</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr"/>
@@ -1631,7 +1639,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>T4-O-DEVE</t>
+          <t>T4-O-DEV</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -1686,7 +1694,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>T4-O-MAND</t>
+          <t>T4-O-LINK</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1711,12 +1719,12 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Mandate</t>
+          <t>Career linkage</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Is that development a prerequisite for promotion, embedded in the promotion course, expected but not mandatory, or unconnected?</t>
+          <t>Where does the link between the development and the transition sit: 4 formally mandated (in policy or embedded in the qualifying course), 3 functionally required (policed, not in policy), 2 expected (self-selected, high uptake), 1 self-selected (uptake by inclination), 0 unconnected?</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1726,12 +1734,12 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Meeting 9 Sep: Not mandated; impression is that all MAJ to LTCOL complete it. Confirm against promotion policy.</t>
-        </is>
-      </c>
-      <c r="J22" s="3" t="inlineStr">
-        <is>
-          <t>STATED 9 SEP</t>
+          <t>Meeting 9 Sep: Level 2, expected: not mandated; impression is that all MAJ to LTCOL complete it. Confirm against promotion policy.</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>TO CONFIRM</t>
         </is>
       </c>
       <c r="K22" s="4" t="inlineStr"/>
@@ -1796,7 +1804,7 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>T4-R-DEVE</t>
+          <t>T4-R-DEV</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
@@ -1851,7 +1859,7 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>T4-R-MAND</t>
+          <t>T4-R-LINK</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
@@ -1876,12 +1884,12 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Mandate</t>
+          <t>Career linkage</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Is that development a prerequisite for promotion, embedded in the promotion course, expected but not mandatory, or unconnected?</t>
+          <t>Where does the link between the development and the transition sit: 4 formally mandated (in policy or embedded in the qualifying course), 3 functionally required (policed, not in policy), 2 expected (self-selected, high uptake), 1 self-selected (uptake by inclination), 0 unconnected?</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -1891,12 +1899,12 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Meeting 9 Sep: Expected for promotion to WO1; 'pretty sure' not mandated in policy; most attend subject to an ILD seat. Confirm against promotion policy.</t>
-        </is>
-      </c>
-      <c r="J25" s="3" t="inlineStr">
-        <is>
-          <t>STATED 9 SEP</t>
+          <t>Meeting 9 Sep: Level 2, expected: expected for promotion to WO1; 'pretty sure' not in policy; most attend subject to an ILD seat. Confirm against promotion policy.</t>
+        </is>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>TO CONFIRM</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr"/>
@@ -1961,7 +1969,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>T5-O-DEVE</t>
+          <t>T5-O-DEV</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
@@ -2016,7 +2024,7 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>T5-O-MAND</t>
+          <t>T5-O-LINK</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
@@ -2041,12 +2049,12 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Mandate</t>
+          <t>Career linkage</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Is that development a prerequisite for promotion, embedded in the promotion course, expected but not mandatory, or unconnected?</t>
+          <t>Where does the link between the development and the transition sit: 4 formally mandated (in policy or embedded in the qualifying course), 3 functionally required (policed, not in policy), 2 expected (self-selected, high uptake), 1 self-selected (uptake by inclination), 0 unconnected?</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -2056,7 +2064,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>Meeting 9 Sep: Mandate not stated; attendance without exception (selected, scrutinised, ambitious).</t>
+          <t>Meeting 9 Sep: Level 2, expected: ILD pathway; attendance without exception (selected, scrutinised, ambitious). Mandate not stated.</t>
         </is>
       </c>
       <c r="J28" s="3" t="inlineStr">
@@ -2126,7 +2134,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>T5-R-DEVE</t>
+          <t>T5-R-DEV</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
@@ -2181,7 +2189,7 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>T5-R-MAND</t>
+          <t>T5-R-LINK</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
@@ -2206,12 +2214,12 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Mandate</t>
+          <t>Career linkage</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Is that development a prerequisite for promotion, embedded in the promotion course, expected but not mandatory, or unconnected?</t>
+          <t>Where does the link between the development and the transition sit: 4 formally mandated (in policy or embedded in the qualifying course), 3 functionally required (policed, not in policy), 2 expected (self-selected, high uptake), 1 self-selected (uptake by inclination), 0 unconnected?</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -2221,7 +2229,7 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>Meeting 9 Sep: Mandate not stated; attendance without exception.</t>
+          <t>Meeting 9 Sep: Level 2, expected: ILD pathway; attendance without exception. Mandate not stated.</t>
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr">
@@ -2291,7 +2299,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>T6-O-DEVE</t>
+          <t>T6-O-DEV</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -2346,7 +2354,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>T6-O-MAND</t>
+          <t>T6-O-LINK</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
@@ -2371,12 +2379,12 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Mandate</t>
+          <t>Career linkage</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Is that development a prerequisite for promotion, embedded in the promotion course, expected but not mandatory, or unconnected?</t>
+          <t>Where does the link between the development and the transition sit: 4 formally mandated (in policy or embedded in the qualifying course), 3 functionally required (policed, not in policy), 2 expected (self-selected, high uptake), 1 self-selected (uptake by inclination), 0 unconnected?</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -2386,7 +2394,7 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>Meeting 9 Sep: Mandate not stated; all complete it well before required.</t>
+          <t>Meeting 9 Sep: Level 2, expected: senior selection pathway; all complete it well before required. Mandate not stated.</t>
         </is>
       </c>
       <c r="J34" s="3" t="inlineStr">
@@ -2456,7 +2464,7 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>T6-R-DEVE</t>
+          <t>T6-R-DEV</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
@@ -2511,7 +2519,7 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>T6-R-MAND</t>
+          <t>T6-R-LINK</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
@@ -2536,12 +2544,12 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Mandate</t>
+          <t>Career linkage</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Is that development a prerequisite for promotion, embedded in the promotion course, expected but not mandatory, or unconnected?</t>
+          <t>Where does the link between the development and the transition sit: 4 formally mandated (in policy or embedded in the qualifying course), 3 functionally required (policed, not in policy), 2 expected (self-selected, high uptake), 1 self-selected (uptake by inclination), 0 unconnected?</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -2551,7 +2559,7 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>Meeting 9 Sep: Mandate not stated; all complete it well before required.</t>
+          <t>Meeting 9 Sep: Level 2, expected: senior selection pathway; all complete it well before required. Mandate not stated.</t>
         </is>
       </c>
       <c r="J37" s="3" t="inlineStr">
@@ -2597,7 +2605,7 @@
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr"/>
-      <c r="J38" s="5" t="inlineStr">
+      <c r="J38" s="6" t="inlineStr">
         <is>
           <t>DATA REQUIRED</t>
         </is>
@@ -2640,7 +2648,7 @@
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr"/>
-      <c r="J39" s="5" t="inlineStr">
+      <c r="J39" s="6" t="inlineStr">
         <is>
           <t>DATA REQUIRED</t>
         </is>
@@ -2683,7 +2691,7 @@
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr"/>
-      <c r="J40" s="5" t="inlineStr">
+      <c r="J40" s="6" t="inlineStr">
         <is>
           <t>DATA REQUIRED</t>
         </is>
@@ -2769,7 +2777,7 @@
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr"/>
-      <c r="J42" s="5" t="inlineStr">
+      <c r="J42" s="6" t="inlineStr">
         <is>
           <t>DATA REQUIRED</t>
         </is>
@@ -2924,133 +2932,157 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A20"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>LDF ALIGNMENT: DATA REQUIRED REGISTER</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr"/>
+      <c r="A2" s="8" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>One row per transition (T1 to T6), per continuum (Officer, Soldier), per fact (promotion point, development intervention, mandate), plus cross-cutting items X1 to X8.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>Populate the three cream columns: Answer, Source cited, Notes. Set Status when done.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr"/>
+      <c r="A5" s="8" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>STATUS VALUES</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>DATA REQUIRED: nothing in hand.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>TO CONFIRM: something in hand but from an estimate (the Leadership Levels poster) or a session document, not authoritative policy.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>STATED 9 SEP: stated at the NZALC meeting of 9 Sep 2026 (Mike and Dave). Treated as the working position; still to be checked against promotion policy or the course data sheet named in the row.</t>
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>STATED 9 SEP: stated at the NZALC meeting of 9 Sep 2026 (Mike and Dave); the transcript governs over the generated notes. Treated as the working position; still to be checked against an authoritative source.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>TO CONFIRM also marks the career-linkage cells where the meeting itself left a question mark or where a policy check decides the state (officer T2 to T4, soldier T3 and T4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>KNOWN: confirmed against an authoritative source.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>NOT APPLICABLE: the category does not apply to this transition for this continuum (state why in Notes).</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="7" t="inlineStr"/>
-    </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>CATEGORY MEANINGS</t>
-        </is>
-      </c>
+      <c r="A13" s="8" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
+          <t>CATEGORY MEANINGS</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
           <t>Promotion point: Which Army promotion or career point corresponds to this LDF transition?</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>Development intervention: Which course or programme develops the individual for this transition (SOLO code, LDS, ELDA, promotion course)?</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t>Mandate: Is that development a prerequisite for promotion, embedded in the promotion course, expected but not mandatory, or unconnected?</t>
-        </is>
-      </c>
-    </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr"/>
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Career linkage: Where does the link between the development and the transition sit: 4 formally mandated (in policy or embedded in the qualifying course), 3 functionally required (policed, not in policy), 2 expected (self-selected, high uptake), 1 self-selected (uptake by inclination), 0 unconnected?</t>
+        </is>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>PRIORITY</t>
-        </is>
-      </c>
+      <c r="A18" s="8" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>The Officer Mandate rows at T2 to T4 decide the piece: confirm the meeting's statements against promotion policy (X1) first.</t>
+          <t>PRIORITY</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="7" t="inlineStr">
-        <is>
-          <t>Then the Soldier Mandate row at T3 (Dave: is ILD LDS Lead Systems a prerequisite in the WO promotion-course CDS?).</t>
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>The Officer Career linkage rows at T2 to T4 decide the piece: confirm the meeting's statements against promotion policy (X1) first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Then the Soldier Career linkage row at T3 (Dave: is ILD LDS Lead Systems a prerequisite in the WO promotion-course CDS?).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>LINKAGE SCALE</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>4 formally mandated; 3 functionally required; 2 expected (high uptake); 1 self-selected (uptake by inclination); 0 unconnected. Record the level in the Answer column once confirmed.</t>
         </is>
       </c>
     </row>

</xml_diff>